<commit_message>
Replaced fn.datetimeparse with fn.datetime
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/odm-v1-to-v2/ids/odm_v1_to_v2_id_code-date.xlsx
+++ b/odm_map/data/modules/odm-v1-to-v2/ids/odm_v1_to_v2_id_code-date.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/data/modules/odm_v1_to_v2/ids/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/odm-v1-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5814FF20-EB08-5A4F-B25A-B43AC55C2CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A95377-60B5-FB4A-B14F-8875A5B2C937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -176,15 +176,6 @@
     <t>reportDate</t>
   </si>
   <si>
-    <t>fn.datetimeparse(dat.samples.__collDT)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.samples.__collDTStart)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.samples.__collDTEnd)</t>
-  </si>
-  <si>
     <t>aDateStart</t>
   </si>
   <si>
@@ -206,21 +197,12 @@
     <t>recDate</t>
   </si>
   <si>
-    <t>fn.datetimeparse(dat.samples.__recDate)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.samples.__lastEdited)</t>
-  </si>
-  <si>
     <t>datasets</t>
   </si>
   <si>
     <t>sentDate</t>
   </si>
   <si>
-    <t>fn.datetimeparse(dat.samples.__sentDate)</t>
-  </si>
-  <si>
     <t>addresses</t>
   </si>
   <si>
@@ -230,61 +212,79 @@
     <t>measureSets</t>
   </si>
   <si>
-    <t>fn.datetimeparse(dat.addresses.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.contacts.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.datasets.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.instruments.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.measures.__aDateStart)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.measures.__aDateEnd)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.measures.__reportDate)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.measures.__relDateStart)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.measures.__relDateEnd)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.measures.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.measureSets.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.organizations.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.polygons.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.protocolRelationships.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.protocols.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.protocolSteps.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.qualityReports.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.sampleRelationships.__lastEdited)</t>
-  </si>
-  <si>
-    <t>fn.datetimeparse(dat.sites.__lastEdited)</t>
+    <t>fn.datetime(dat.addresses.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.contacts.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.datasets.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.instruments.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.measures.__aDateStart)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.measures.__aDateEnd)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.measures.__reportDate)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.measures.__relDateStart)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.measures.__relDateEnd)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.measures.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.measureSets.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.organizations.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.polygons.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.protocolRelationships.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.protocols.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.protocolSteps.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.qualityReports.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.sampleRelationships.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.samples.__collDT)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.samples.__collDTStart)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.samples.__collDTEnd)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.samples.__sentDate)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.samples.__recDate)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.samples.__lastEdited)</t>
+  </si>
+  <si>
+    <t>fn.datetime(dat.sites.__lastEdited)</t>
   </si>
 </sst>
 </file>
@@ -360,9 +360,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -400,7 +400,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -506,7 +506,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -648,7 +648,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -680,13 +680,13 @@
     </row>
     <row r="2" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -706,21 +706,21 @@
         <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -740,10 +740,10 @@
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -787,10 +787,10 @@
         <v>0</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -798,10 +798,10 @@
         <v>0</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -812,7 +812,7 @@
         <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -820,10 +820,10 @@
         <v>0</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -831,10 +831,10 @@
         <v>0</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -842,21 +842,21 @@
         <v>0</v>
       </c>
       <c r="B20" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B22" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C22" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -876,10 +876,10 @@
         <v>20</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C25" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -898,21 +898,21 @@
         <v>21</v>
       </c>
       <c r="B28" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C28" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B30" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C30" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -931,10 +931,10 @@
         <v>22</v>
       </c>
       <c r="B33" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C33" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
@@ -953,10 +953,10 @@
         <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C36" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
@@ -989,21 +989,21 @@
         <v>2</v>
       </c>
       <c r="B40" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C40" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B42" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C42" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1037,7 +1037,7 @@
         <v>40</v>
       </c>
       <c r="C46" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
@@ -1048,7 +1048,7 @@
         <v>41</v>
       </c>
       <c r="C47" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
@@ -1059,7 +1059,7 @@
         <v>42</v>
       </c>
       <c r="C48" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -1067,10 +1067,10 @@
         <v>23</v>
       </c>
       <c r="B49" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C49" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -1078,10 +1078,10 @@
         <v>23</v>
       </c>
       <c r="B50" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C50" t="s">
-        <v>54</v>
+        <v>78</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -1089,10 +1089,10 @@
         <v>23</v>
       </c>
       <c r="B51" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C51" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -1111,7 +1111,7 @@
         <v>24</v>
       </c>
       <c r="B54" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C54" t="s">
         <v>80</v>

</xml_diff>